<commit_message>
docs: precio PRO fijo en S/89 y video rewarded fuera del modelo
El video rewarded se retira: AdMob exige app nativa y Gatekeeper es solo
plataforma web, asi que no es una via disponible. Quedan banner web y
patrocinio local.

El plan PRO queda definido en S/89/mes; la tabla de sensibilidad de precio se
conserva solo como referencia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Gatekeeper_Modelo_2Planes.xlsx
+++ b/docs/Gatekeeper_Modelo_2Planes.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -802,7 +802,7 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Plan único. Ver sensibilidad de precio en la hoja 5.</t>
+          <t>PLAN ÚNICO DEFINIDO: S/ 89/mes. La hoja 5 solo muestra sensibilidad.</t>
         </is>
       </c>
     </row>
@@ -969,20 +969,20 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Vía activa (1=Banner / 2=Video / 3=Patrocinio)</t>
+          <t>Vía activa (1=Banner / 2=Patrocinio)</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>1, 2 ó 3</t>
+          <t>1 ó 2</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Elige cuál de las tres vías estás usando.</t>
+          <t>El video rewarded NO aplica: exige app nativa y Gatekeeper es solo web.</t>
         </is>
       </c>
     </row>
@@ -1009,131 +1009,131 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>CPM video rewarded</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="n">
-        <v>3</v>
+          <t>Patrocinio local — por espacio</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>80</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>S/ /mes</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Rango 2 – 5. Requiere app nativa (ver hoja 4).</t>
+          <t>Venta directa a un comercio de la zona.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Patrocinio local — por espacio</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>80</v>
+          <t>Patrocinadores vendidos</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>S/ /mes</t>
+          <t>espacios</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Venta directa a un comercio de la zona.</t>
+          <t>Cuántos espacios tienes colocados.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Patrocinadores vendidos</t>
+          <t>Impresiones por residente / mes</t>
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>espacios</t>
+          <t>impresiones</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Cuántos espacios tienes colocados.</t>
+          <t>≈ 4 sesiones × 3 vistas.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Impresiones por residente / mes</t>
-        </is>
-      </c>
-      <c r="B29" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>impresiones</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>≈ 4 sesiones × 3 vistas.</t>
-        </is>
-      </c>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Motor de conversión (así el GRATIS genera ingresos)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Motor de conversión (así el GRATIS genera ingresos)</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Tasa de conversión GRATIS → PRO</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>De cada 100 cuentas gratis, cuántas terminan pagando.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>Tasa de conversión GRATIS → PRO</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>De cada 100 cuentas gratis, cuántas terminan pagando.</t>
-        </is>
-      </c>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Estructura del negocio</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Estructura del negocio</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Tu sueldo</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>S/ /mes</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>El mayor costo fijo. Es tu decisión.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Tu sueldo</t>
+          <t>Marketing pagado</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
@@ -1142,18 +1142,18 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>El mayor costo fijo. Es tu decisión.</t>
+          <t>Limitado: el canal principal es el plan gratis.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Marketing pagado</t>
+          <t>Soporte — valor imputado</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
@@ -1161,26 +1161,6 @@
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Limitado: el canal principal es el plan gratis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>Soporte — valor imputado</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>S/ /mes</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>0 = lo das tú y no lo cobras. NO sale del banco.</t>
         </is>
@@ -1834,7 +1814,7 @@
         </is>
       </c>
       <c r="B12" s="25">
-        <f>'1. Supuestos'!$B$29/1000*'1. Supuestos'!$B$25*'1. Supuestos'!$B$6*'1. Supuestos'!$B$18</f>
+        <f>'1. Supuestos'!$B$28/1000*'1. Supuestos'!$B$25*'1. Supuestos'!$B$6*'1. Supuestos'!$B$18</f>
         <v/>
       </c>
       <c r="C12" s="27">
@@ -1854,15 +1834,15 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2. Video rewarded (AdMob)</t>
+          <t>2. Patrocinio local directo</t>
         </is>
       </c>
       <c r="B13" s="25">
-        <f>'1. Supuestos'!$B$29/1000*'1. Supuestos'!$B$26*'1. Supuestos'!$B$6*'1. Supuestos'!$B$18</f>
+        <f>'1. Supuestos'!$B$26*'1. Supuestos'!$B$27</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>B13*'1. Supuestos'!$B$20</f>
+        <f>B13</f>
         <v/>
       </c>
       <c r="D13" s="28">
@@ -1871,294 +1851,277 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>REQUIERE APP — Es la de mayor ingreso, pero AdMob exige app nativa y Gatekeeper es web/PWA. Habría que empaquetarla para Play Store primero.</t>
+          <t>SIN RIESGO — Sin ad network, sin scripts, sin tracking, CSP intacto. Contra: es venta 1-a-1 tuya, no ingreso pasivo.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>3. Patrocinio local directo</t>
-        </is>
-      </c>
-      <c r="B14" s="25">
-        <f>'1. Supuestos'!$B$27*'1. Supuestos'!$B$28</f>
-        <v/>
-      </c>
-      <c r="C14" s="27">
-        <f>B14</f>
-        <v/>
-      </c>
-      <c r="D14" s="28">
-        <f>IF(C14&gt;='4. Plan GRATIS'!$B$8,"SÍ","NO")</f>
-        <v/>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>SIN RIESGO — Sin ad network, sin scripts, sin tracking, CSP intacto. Contra: es venta 1-a-1 tuya, no ingreso pasivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>El patrocinio es un monto fijo total (no por cuenta); las otras dos escalan con tu base gratis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>El patrocinio es un monto fijo total (no por cuenta); el banner escala con tu base gratis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>INGRESO PUBLICITARIO SEGÚN LA VÍA QUE ELEGISTE</t>
         </is>
       </c>
-      <c r="B17" s="30">
-        <f>'1. Supuestos'!$B$23*CHOOSE('1. Supuestos'!$B$24,C12,C13,C14)</f>
-        <v/>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="B16" s="30">
+        <f>'1. Supuestos'!$B$23*CHOOSE('1. Supuestos'!$B$24,C12,C13)</f>
+        <v/>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Cambia 'Vía activa' en la hoja 1 para comparar. Con 0 en 'Activar publicidad' se apaga.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>C) VÍA 2 — CONVERSIÓN A PRO (aquí está el ingreso de verdad)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Tasa de conversión gratis → PRO</t>
+        </is>
+      </c>
+      <c r="B20" s="31">
+        <f>'1. Supuestos'!$B$30</f>
+        <v/>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>De cada 100 cuentas gratis, cuántas terminan pagando.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Tasa de conversión gratis → PRO</t>
-        </is>
-      </c>
-      <c r="B21" s="31">
-        <f>'1. Supuestos'!$B$31</f>
+          <t>Clientes PRO que produce tu base gratis</t>
+        </is>
+      </c>
+      <c r="B21" s="21">
+        <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$30,0)</f>
         <v/>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>clientes</t>
         </is>
       </c>
       <c r="D21" s="24" t="n"/>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>De cada 100 cuentas gratis, cuántas terminan pagando.</t>
+          <t>Cuentas gratis × tasa de conversión.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Clientes PRO que produce tu base gratis</t>
-        </is>
-      </c>
-      <c r="B22" s="21">
-        <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$31,0)</f>
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>INGRESO POR CONVERSIÓN</t>
+        </is>
+      </c>
+      <c r="B22" s="26">
+        <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$30,0)*'5. Plan PRO'!$B$12</f>
         <v/>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>clientes</t>
+          <t>S/ /mes</t>
         </is>
       </c>
       <c r="D22" s="24" t="n"/>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Cuentas gratis × tasa de conversión.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="22" t="inlineStr">
-        <is>
-          <t>INGRESO POR CONVERSIÓN</t>
-        </is>
-      </c>
-      <c r="B23" s="26">
-        <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$31,0)*'5. Plan PRO'!$B$12</f>
-        <v/>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
+          <t>Clientes convertidos × contribución de cada uno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>D) BALANCE DEL PLAN GRATIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Clientes convertidos × contribución de cada uno.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>D) BALANCE DEL PLAN GRATIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>S/ /mes</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr"/>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Lectura</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>(+) Ingreso por publicidad</t>
+        </is>
+      </c>
+      <c r="B26" s="25">
+        <f>'4. Plan GRATIS'!$B$16</f>
+        <v/>
+      </c>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Directo, si la activas.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>(+) Ingreso por publicidad</t>
+          <t>(+) Ingreso por conversión a PRO</t>
         </is>
       </c>
       <c r="B27" s="25">
-        <f>'4. Plan GRATIS'!$B$17</f>
+        <f>'4. Plan GRATIS'!$B$22</f>
         <v/>
       </c>
       <c r="C27" s="24" t="n"/>
       <c r="D27" s="24" t="n"/>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Directo, si la activas.</t>
+          <t>Indirecto, pero es el grande.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>(+) Ingreso por conversión a PRO</t>
+          <t>(–) Costo de la base gratis</t>
         </is>
       </c>
       <c r="B28" s="25">
-        <f>'4. Plan GRATIS'!$B$23</f>
+        <f>-'4. Plan GRATIS'!$B$8</f>
         <v/>
       </c>
       <c r="C28" s="24" t="n"/>
       <c r="D28" s="24" t="n"/>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Indirecto, pero es el grande.</t>
+          <t>Lo que te cuesta servirla.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>(–) Costo de la base gratis</t>
-        </is>
-      </c>
-      <c r="B29" s="25">
-        <f>-'4. Plan GRATIS'!$B$8</f>
-        <v/>
-      </c>
-      <c r="C29" s="24" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>Lo que te cuesta servirla.</t>
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>RESULTADO NETO DEL PLAN GRATIS</t>
+        </is>
+      </c>
+      <c r="B29" s="26">
+        <f>SUM(B26:B28)</f>
+        <v/>
+      </c>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>Si es positivo, el plan gratis GANA dinero.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>RESULTADO NETO DEL PLAN GRATIS</t>
-        </is>
-      </c>
-      <c r="B30" s="26">
-        <f>SUM(B27:B29)</f>
-        <v/>
-      </c>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="inlineStr">
-        <is>
-          <t>Si es positivo, el plan gratis GANA dinero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>Retorno por cada sol invertido en el gratis</t>
         </is>
       </c>
-      <c r="B31" s="32">
-        <f>('4. Plan GRATIS'!$B$17+'4. Plan GRATIS'!$B$23)/'4. Plan GRATIS'!$B$8</f>
-        <v/>
-      </c>
-      <c r="C31" s="24" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="B30" s="32">
+        <f>('4. Plan GRATIS'!$B$16+'4. Plan GRATIS'!$B$22)/'4. Plan GRATIS'!$B$8</f>
+        <v/>
+      </c>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Cuántas veces recuperas lo que gastas en regalar el producto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>• Respuesta a '¿cómo genero ingresos en el plan gratis?': por conversión. La publicidad es el extra, no el motor.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>• Respuesta a '¿cómo genero ingresos en el plan gratis?': por conversión. La publicidad es el extra, no el motor.</t>
+          <t>• Con 100 cuentas gratis y 5% de conversión obtienes 5 clientes PRO. Eso vale mucho más que cualquier CPM.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>• Con 100 cuentas gratis y 5% de conversión obtienes 5 clientes PRO. Eso vale mucho más que cualquier CPM.</t>
+          <t>• Si subes la conversión del 5% al 8%, ganas más que activando publicidad. Optimiza eso primero.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>• Si subes la conversión del 5% al 8%, ganas más que activando publicidad. Optimiza eso primero.</t>
+          <t>• El video rewarded queda descartado por arquitectura: AdMob exige app nativa y Gatekeeper es solo web.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>• La publicidad SÍ cubre el costo del gratis — el problema nunca fue el dinero, es qué le hace al producto.</t>
+          <t>• El banner SÍ cubre el costo del gratis. La decisión no es de dinero, es qué le hace al producto y al CSP.</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2276,7 @@
         </is>
       </c>
       <c r="B10" s="25">
-        <f>-'1. Supuestos'!$B$35</f>
+        <f>-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
       <c r="C10" s="24" t="n"/>
@@ -2413,7 +2376,7 @@
         <v>49</v>
       </c>
       <c r="B17" s="25">
-        <f>A17/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A17*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$35</f>
+        <f>A17/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A17*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
       <c r="C17" s="35">
@@ -2435,7 +2398,7 @@
         <v>69</v>
       </c>
       <c r="B18" s="25">
-        <f>A18/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A18*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$35</f>
+        <f>A18/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A18*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
       <c r="C18" s="35">
@@ -2457,7 +2420,7 @@
         <v>89</v>
       </c>
       <c r="B19" s="25">
-        <f>A19/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A19*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$35</f>
+        <f>A19/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A19*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
       <c r="C19" s="35">
@@ -2479,7 +2442,7 @@
         <v>99</v>
       </c>
       <c r="B20" s="25">
-        <f>A20/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A20*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$35</f>
+        <f>A20/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A20*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
       <c r="C20" s="35">
@@ -2501,7 +2464,7 @@
         <v>129</v>
       </c>
       <c r="B21" s="25">
-        <f>A21/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A21*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$35</f>
+        <f>A21/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A21*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
       <c r="C21" s="35">
@@ -2611,7 +2574,7 @@
         </is>
       </c>
       <c r="B6" s="36">
-        <f>'1. Supuestos'!$B$33</f>
+        <f>'1. Supuestos'!$B$32</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n"/>
@@ -2629,7 +2592,7 @@
         </is>
       </c>
       <c r="B7" s="36">
-        <f>'1. Supuestos'!$B$34</f>
+        <f>'1. Supuestos'!$B$33</f>
         <v/>
       </c>
       <c r="C7" s="24" t="n"/>
@@ -2661,7 +2624,7 @@
         </is>
       </c>
       <c r="B9" s="36">
-        <f>'4. Plan GRATIS'!$B$17</f>
+        <f>'4. Plan GRATIS'!$B$16</f>
         <v/>
       </c>
       <c r="C9" s="24" t="n"/>
@@ -2767,7 +2730,7 @@
         </is>
       </c>
       <c r="B16" s="21">
-        <f>ROUNDUP(ROUNDUP(B10/'5. Plan PRO'!$B$12,0)/'1. Supuestos'!$B$31,0)</f>
+        <f>ROUNDUP(ROUNDUP(B10/'5. Plan PRO'!$B$12,0)/'1. Supuestos'!$B$30,0)</f>
         <v/>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -2789,7 +2752,7 @@
         </is>
       </c>
       <c r="B17" s="21">
-        <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$31,0)</f>
+        <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$30,0)</f>
         <v/>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -2841,7 +2804,7 @@
         </is>
       </c>
       <c r="B21" s="27">
-        <f>'4. Plan GRATIS'!$B$17</f>
+        <f>'4. Plan GRATIS'!$B$16</f>
         <v/>
       </c>
       <c r="C21" s="40">
@@ -2851,7 +2814,7 @@
       <c r="D21" s="24" t="n"/>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Ingreso directo, escala con tu base gratis.</t>
+          <t>Ingreso directo. Con banner escala con tu base gratis.</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2825,7 @@
         </is>
       </c>
       <c r="B22" s="27">
-        <f>'4. Plan GRATIS'!$B$23</f>
+        <f>'4. Plan GRATIS'!$B$22</f>
         <v/>
       </c>
       <c r="C22" s="40">

</xml_diff>

<commit_message>
docs: uso realista en el modelo y techo del plan ilimitado
- Las visitas por residente del plan Pro pasan de 4 a 8 al mes (dos por
  semana). Cuatro se quedaba corto.
- Se aclara en los supuestos que los 30 residentes y las visitas por
  residente NO son limites del plan: Pro es ilimitado. Son el tamano y el
  uso promedio con los que se estiman los costos.
- Nueva seccion en la hoja del plan Pro: que queda de los S/89 segun el
  tamano del cliente (de 15 a 1.000 residentes) y a partir de cuantos
  residentes un cliente dejaria de ser rentable.
- Se eliminan las columnas vacias que quedaban en las hojas 4, 5 y 6.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Gatekeeper_Modelo_2Planes.xlsx
+++ b/docs/Gatekeeper_Modelo_2Planes.xlsx
@@ -66,7 +66,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +103,11 @@
         <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -130,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,7 +184,6 @@
     <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -202,6 +206,7 @@
     <xf numFmtId="169" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -212,6 +217,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -822,7 +830,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Promedio de un condominio real.</t>
+          <t>⚠️ NO es un límite: PRO es ilimitado. Es el TAMAÑO PROMEDIO de un cliente, para estimar costos.</t>
         </is>
       </c>
     </row>
@@ -833,7 +841,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
@@ -842,7 +850,7 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>≈ 1 por semana.</t>
+          <t>≈ 2 por semana. Tampoco es un límite: es uso promedio estimado.</t>
         </is>
       </c>
     </row>
@@ -872,7 +880,7 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Tope del plan gratuito.</t>
+          <t>Este SÍ es un límite real del plan gratuito.</t>
         </is>
       </c>
     </row>
@@ -892,7 +900,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Menor uso: es de prueba.</t>
+          <t>Menor uso: el gratis se prueba, no se opera a full.</t>
         </is>
       </c>
     </row>
@@ -1659,8 +1667,8 @@
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1700,8 +1708,7 @@
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -1722,8 +1729,7 @@
           <t>cuentas</t>
         </is>
       </c>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Editable en la hoja 1.</t>
         </is>
@@ -1735,7 +1741,7 @@
           <t>Costo por cuenta gratis</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="24">
         <f>'3. Costos x Usuario'!$B$13</f>
         <v/>
       </c>
@@ -1744,8 +1750,7 @@
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>15 residentes × costo por residente.</t>
         </is>
@@ -1757,7 +1762,7 @@
           <t>COSTO TOTAL DE TU BASE GRATIS</t>
         </is>
       </c>
-      <c r="B8" s="26">
+      <c r="B8" s="25">
         <f>'1. Supuestos'!$B$20*'3. Costos x Usuario'!$B$13</f>
         <v/>
       </c>
@@ -1766,8 +1771,7 @@
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Este es el gasto real de regalar el producto.</t>
         </is>
@@ -1813,15 +1817,15 @@
           <t>1. Banner display (AdSense web)</t>
         </is>
       </c>
-      <c r="B12" s="25">
+      <c r="B12" s="24">
         <f>'1. Supuestos'!$B$28/1000*'1. Supuestos'!$B$25*'1. Supuestos'!$B$6*'1. Supuestos'!$B$18</f>
         <v/>
       </c>
-      <c r="C12" s="27">
+      <c r="C12" s="26">
         <f>B12*'1. Supuestos'!$B$20</f>
         <v/>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="27">
         <f>IF(C12&gt;='4. Plan GRATIS'!$B$8,"SÍ","NO")</f>
         <v/>
       </c>
@@ -1837,15 +1841,15 @@
           <t>2. Patrocinio local directo</t>
         </is>
       </c>
-      <c r="B13" s="25">
+      <c r="B13" s="24">
         <f>'1. Supuestos'!$B$26*'1. Supuestos'!$B$27</f>
         <v/>
       </c>
-      <c r="C13" s="27">
+      <c r="C13" s="26">
         <f>B13</f>
         <v/>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="27">
         <f>IF(C13&gt;='4. Plan GRATIS'!$B$8,"SÍ","NO")</f>
         <v/>
       </c>
@@ -1863,12 +1867,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>INGRESO PUBLICITARIO SEGÚN LA VÍA QUE ELEGISTE</t>
         </is>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="29">
         <f>'1. Supuestos'!$B$23*CHOOSE('1. Supuestos'!$B$24,C12,C13)</f>
         <v/>
       </c>
@@ -1901,8 +1905,7 @@
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -1914,7 +1917,7 @@
           <t>Tasa de conversión gratis → PRO</t>
         </is>
       </c>
-      <c r="B20" s="31">
+      <c r="B20" s="30">
         <f>'1. Supuestos'!$B$30</f>
         <v/>
       </c>
@@ -1923,8 +1926,7 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>De cada 100 cuentas gratis, cuántas terminan pagando.</t>
         </is>
@@ -1945,8 +1947,7 @@
           <t>clientes</t>
         </is>
       </c>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Cuentas gratis × tasa de conversión.</t>
         </is>
@@ -1958,7 +1959,7 @@
           <t>INGRESO POR CONVERSIÓN</t>
         </is>
       </c>
-      <c r="B22" s="26">
+      <c r="B22" s="25">
         <f>ROUND('1. Supuestos'!$B$20*'1. Supuestos'!$B$30,0)*'5. Plan PRO'!$B$12</f>
         <v/>
       </c>
@@ -1967,8 +1968,7 @@
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Clientes convertidos × contribución de cada uno.</t>
         </is>
@@ -1992,9 +1992,7 @@
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Lectura</t>
         </is>
@@ -2006,13 +2004,11 @@
           <t>(+) Ingreso por publicidad</t>
         </is>
       </c>
-      <c r="B26" s="25">
+      <c r="B26" s="24">
         <f>'4. Plan GRATIS'!$B$16</f>
         <v/>
       </c>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Directo, si la activas.</t>
         </is>
@@ -2024,13 +2020,11 @@
           <t>(+) Ingreso por conversión a PRO</t>
         </is>
       </c>
-      <c r="B27" s="25">
+      <c r="B27" s="24">
         <f>'4. Plan GRATIS'!$B$22</f>
         <v/>
       </c>
-      <c r="C27" s="24" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Indirecto, pero es el grande.</t>
         </is>
@@ -2042,13 +2036,11 @@
           <t>(–) Costo de la base gratis</t>
         </is>
       </c>
-      <c r="B28" s="25">
+      <c r="B28" s="24">
         <f>-'4. Plan GRATIS'!$B$8</f>
         <v/>
       </c>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Lo que te cuesta servirla.</t>
         </is>
@@ -2060,13 +2052,11 @@
           <t>RESULTADO NETO DEL PLAN GRATIS</t>
         </is>
       </c>
-      <c r="B29" s="26">
+      <c r="B29" s="25">
         <f>SUM(B26:B28)</f>
         <v/>
       </c>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Si es positivo, el plan gratis GANA dinero.</t>
         </is>
@@ -2078,13 +2068,11 @@
           <t>Retorno por cada sol invertido en el gratis</t>
         </is>
       </c>
-      <c r="B30" s="32">
+      <c r="B30" s="31">
         <f>('4. Plan GRATIS'!$B$16+'4. Plan GRATIS'!$B$22)/'4. Plan GRATIS'!$B$8</f>
         <v/>
       </c>
-      <c r="C30" s="24" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Cuántas veces recuperas lo que gastas en regalar el producto.</t>
         </is>
@@ -2136,14 +2124,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2171,13 +2157,13 @@
           <t>Importe</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
+      <c r="D4" s="32" t="n"/>
+      <c r="E4" s="32" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2185,17 +2171,17 @@
           <t>Precio de lista</t>
         </is>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="24">
         <f>'1. Supuestos'!$B$14</f>
         <v/>
       </c>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Lo que ve el cliente.</t>
         </is>
       </c>
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="32" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2203,17 +2189,17 @@
           <t>(–) IGV incluido</t>
         </is>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="24">
         <f>-('1. Supuestos'!$B$14-'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7))</f>
         <v/>
       </c>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Va a SUNAT, no es tuyo.</t>
         </is>
       </c>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="32" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2221,17 +2207,17 @@
           <t>(=) Ingreso neto</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="24">
         <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)</f>
         <v/>
       </c>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Lo que factura el negocio.</t>
         </is>
       </c>
+      <c r="D7" s="32" t="n"/>
+      <c r="E7" s="32" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2239,17 +2225,17 @@
           <t>(–) Comisión de pasarela</t>
         </is>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="24">
         <f>-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)</f>
         <v/>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Con transferencia/Yape esto es CERO.</t>
         </is>
       </c>
+      <c r="D8" s="32" t="n"/>
+      <c r="E8" s="32" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2257,17 +2243,17 @@
           <t>(–) Costo de servirlo</t>
         </is>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="24">
         <f>-'3. Costos x Usuario'!$C$13</f>
         <v/>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Infraestructura de sus 30 residentes.</t>
         </is>
       </c>
+      <c r="D9" s="32" t="n"/>
+      <c r="E9" s="32" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2275,17 +2261,17 @@
           <t>(–) Soporte imputado</t>
         </is>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="24">
         <f>-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>En 0: lo das tú y no lo cobras.</t>
         </is>
       </c>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="32" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
@@ -2293,17 +2279,17 @@
           <t>CONTRIBUCIÓN POR CLIENTE / MES</t>
         </is>
       </c>
-      <c r="B11" s="26">
+      <c r="B11" s="25">
         <f>B5+B6+B8+B9+B10</f>
         <v/>
       </c>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Lo que aporta cada cliente a cubrir tus costos fijos.</t>
         </is>
       </c>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="32" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -2311,17 +2297,17 @@
           <t>Contribución (referencia interna)</t>
         </is>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="26">
         <f>B11</f>
         <v/>
       </c>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Celda que usan las hojas 4 y 6. No la muevas.</t>
         </is>
       </c>
+      <c r="D12" s="32" t="n"/>
+      <c r="E12" s="32" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
@@ -2333,9 +2319,9 @@
         <f>B11/B5</f>
         <v/>
       </c>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="24" t="n"/>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
@@ -2375,7 +2361,7 @@
       <c r="A17" s="34" t="n">
         <v>49</v>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="24">
         <f>A17/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A17*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
@@ -2397,7 +2383,7 @@
       <c r="A18" s="34" t="n">
         <v>69</v>
       </c>
-      <c r="B18" s="25">
+      <c r="B18" s="24">
         <f>A18/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A18*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
@@ -2419,7 +2405,7 @@
       <c r="A19" s="34" t="n">
         <v>89</v>
       </c>
-      <c r="B19" s="25">
+      <c r="B19" s="24">
         <f>A19/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A19*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
@@ -2441,7 +2427,7 @@
       <c r="A20" s="34" t="n">
         <v>99</v>
       </c>
-      <c r="B20" s="25">
+      <c r="B20" s="24">
         <f>A20/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A20*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
@@ -2463,7 +2449,7 @@
       <c r="A21" s="34" t="n">
         <v>129</v>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="24">
         <f>A21/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,(A21*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-'3. Costos x Usuario'!$C$13-'1. Supuestos'!$B$34</f>
         <v/>
       </c>
@@ -2492,6 +2478,229 @@
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>• Cobrar ANUAL por transferencia elimina la comisión completa y te paga 12 meses por adelantado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>¿HASTA DÓNDE AGUANTA EL PLAN ILIMITADO?</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>El único costo que crece con el tamaño del cliente son los correos de aviso. Esta tabla muestra qué queda de los S/ 89 según cuántos residentes tenga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Tamaño del cliente</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Correos al mes</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Costo de correos</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Contribución</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>15 residentes</t>
+        </is>
+      </c>
+      <c r="B29" s="21">
+        <f>15*'1. Supuestos'!$B$16*2</f>
+        <v/>
+      </c>
+      <c r="C29" s="24">
+        <f>15*'1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6</f>
+        <v/>
+      </c>
+      <c r="D29" s="26">
+        <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="30">
+        <f>D29/'1. Supuestos'!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>30 residentes</t>
+        </is>
+      </c>
+      <c r="B30" s="21">
+        <f>30*'1. Supuestos'!$B$16*2</f>
+        <v/>
+      </c>
+      <c r="C30" s="24">
+        <f>30*'1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6</f>
+        <v/>
+      </c>
+      <c r="D30" s="26">
+        <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="30">
+        <f>D30/'1. Supuestos'!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>100 residentes</t>
+        </is>
+      </c>
+      <c r="B31" s="21">
+        <f>100*'1. Supuestos'!$B$16*2</f>
+        <v/>
+      </c>
+      <c r="C31" s="24">
+        <f>100*'1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6</f>
+        <v/>
+      </c>
+      <c r="D31" s="26">
+        <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="30">
+        <f>D31/'1. Supuestos'!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>300 residentes</t>
+        </is>
+      </c>
+      <c r="B32" s="21">
+        <f>300*'1. Supuestos'!$B$16*2</f>
+        <v/>
+      </c>
+      <c r="C32" s="24">
+        <f>300*'1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6</f>
+        <v/>
+      </c>
+      <c r="D32" s="26">
+        <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="30">
+        <f>D32/'1. Supuestos'!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>500 residentes</t>
+        </is>
+      </c>
+      <c r="B33" s="21">
+        <f>500*'1. Supuestos'!$B$16*2</f>
+        <v/>
+      </c>
+      <c r="C33" s="24">
+        <f>500*'1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6</f>
+        <v/>
+      </c>
+      <c r="D33" s="26">
+        <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="30">
+        <f>D33/'1. Supuestos'!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>1.000 residentes</t>
+        </is>
+      </c>
+      <c r="B34" s="21">
+        <f>1000*'1. Supuestos'!$B$16*2</f>
+        <v/>
+      </c>
+      <c r="C34" s="24">
+        <f>1000*'1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6</f>
+        <v/>
+      </c>
+      <c r="D34" s="26">
+        <f>'1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0)-C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="30">
+        <f>D34/'1. Supuestos'!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>Residentes necesarios para que un cliente deje de ser rentable</t>
+        </is>
+      </c>
+      <c r="B36" s="37">
+        <f>ROUND(('1. Supuestos'!$B$14/(1+'1. Supuestos'!$B$7)-IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11),0))/('1. Supuestos'!$B$16*2*0.0004*'1. Supuestos'!$B$6),0)</f>
+        <v/>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Un condominio grande en Perú tiene 200-500 residentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• ⚠️ Los 30 residentes y las visitas por residente de la hoja 1 NO son límites del plan: son el uso PROMEDIO con el que se estiman los costos. PRO es ilimitado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>• El riesgo del "ilimitado" no es el costo de servidor: es el soporte. Y hoy lo das tú sin cobrarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>• Límite operativo a vigilar: Resend Pro son 50.000 correos al mes. Con clientes de 300 residentes caben unos 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>• Por eso conviene un fair-use de visitas en el contrato: no por dinero, sino para poder decir que no ante un abuso.</t>
         </is>
       </c>
     </row>
@@ -2506,14 +2715,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2541,9 +2748,7 @@
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -2559,9 +2764,7 @@
         <f>'2. Infraestructura'!$D$11</f>
         <v/>
       </c>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Vercel + Neon + dominio.</t>
         </is>
@@ -2577,9 +2780,7 @@
         <f>'1. Supuestos'!$B$32</f>
         <v/>
       </c>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>El componente más grande de tu estructura.</t>
         </is>
@@ -2595,9 +2796,7 @@
         <f>'1. Supuestos'!$B$33</f>
         <v/>
       </c>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Limitado a propósito.</t>
         </is>
@@ -2609,13 +2808,11 @@
           <t>TOTAL COSTOS FIJOS</t>
         </is>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="38">
         <f>SUM(B5:B7)</f>
         <v/>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
+      <c r="C8" s="32" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2627,9 +2824,7 @@
         <f>'4. Plan GRATIS'!$B$16</f>
         <v/>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Si activaste publicidad, reduce lo que deben cubrir las suscripciones.</t>
         </is>
@@ -2641,13 +2836,11 @@
           <t>NETO A CUBRIR CON SUSCRIPCIONES</t>
         </is>
       </c>
-      <c r="B10" s="38">
+      <c r="B10" s="39">
         <f>MAX(0,B8-B9)</f>
         <v/>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="24" t="n"/>
+      <c r="C10" s="32" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -2672,8 +2865,7 @@
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Lectura</t>
         </is>
@@ -2685,7 +2877,7 @@
           <t>CLIENTES PRO NECESARIOS</t>
         </is>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="40">
         <f>ROUNDUP(B10/'5. Plan PRO'!$B$12,0)</f>
         <v/>
       </c>
@@ -2694,8 +2886,7 @@
           <t>clientes</t>
         </is>
       </c>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Este es tu número. Todo lo demás es ruido.</t>
         </is>
@@ -2716,8 +2907,7 @@
           <t>S/ /mes</t>
         </is>
       </c>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Lo que verías entrar por suscripciones.</t>
         </is>
@@ -2738,8 +2928,7 @@
           <t>cuentas</t>
         </is>
       </c>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Si TODOS tus clientes vinieran del plan gratis, esta es la base que necesitas.</t>
         </is>
@@ -2760,8 +2949,7 @@
           <t>clientes</t>
         </is>
       </c>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Compara contra los clientes necesarios: te dice cuánto te falta.</t>
         </is>
@@ -2790,8 +2978,7 @@
           <t>Equivale a</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Comentario</t>
         </is>
@@ -2803,16 +2990,15 @@
           <t>Publicidad en el gratis (vía elegida)</t>
         </is>
       </c>
-      <c r="B21" s="27">
+      <c r="B21" s="26">
         <f>'4. Plan GRATIS'!$B$16</f>
         <v/>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="41">
         <f>B21/'5. Plan PRO'!$B$12</f>
         <v/>
       </c>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Ingreso directo. Con banner escala con tu base gratis.</t>
         </is>
@@ -2824,16 +3010,15 @@
           <t>Conversión gratis → PRO</t>
         </is>
       </c>
-      <c r="B22" s="27">
+      <c r="B22" s="26">
         <f>'4. Plan GRATIS'!$B$22</f>
         <v/>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="41">
         <f>B22/'5. Plan PRO'!$B$12</f>
         <v/>
       </c>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>El motor real del negocio.</t>
         </is>
@@ -2845,16 +3030,15 @@
           <t>Quitar la pasarela (cobro anual)</t>
         </is>
       </c>
-      <c r="B23" s="27">
+      <c r="B23" s="26">
         <f>IF('1. Supuestos'!$B$12=1,('1. Supuestos'!$B$14*'1. Supuestos'!$B$9+'1. Supuestos'!$B$10*'1. Supuestos'!$B$6)*(1+'1. Supuestos'!$B$11)*ROUNDUP(B10/'5. Plan PRO'!$B$12,0),0)</f>
         <v/>
       </c>
-      <c r="C23" s="40">
+      <c r="C23" s="41">
         <f>B23/'5. Plan PRO'!$B$12</f>
         <v/>
       </c>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Ahorro inmediato, sin vender nada más.</t>
         </is>

</xml_diff>